<commit_message>
Minor tweaks to restart the conversion to multiple pathogens.
</commit_message>
<xml_diff>
--- a/patchr/resources/PLATES_v2.0.0/AB[BATCH_ID].4RVP.xlsx
+++ b/patchr/resources/PLATES_v2.0.0/AB[BATCH_ID].4RVP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/PLATES_v2.0.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97FA572C-A40B-B641-8FA4-C55190B229CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6CD220-FDCE-6B4A-B5E3-EDDBFD0C062E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43840" yWindow="4060" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="6" r:id="rId1"/>
@@ -1761,7 +1761,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="46" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C5" s="42"/>
       <c r="D5" s="42"/>
@@ -2210,7 +2210,7 @@
         <v>117</v>
       </c>
       <c r="B19" s="52" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C19"/>
     </row>
@@ -2426,7 +2426,7 @@
         <v>93</v>
       </c>
       <c r="B28" s="59" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C28"/>
       <c r="D28" s="42"/>
@@ -2458,7 +2458,7 @@
         <v>77</v>
       </c>
       <c r="B29" s="60" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C29"/>
       <c r="D29" s="42"/>

</xml_diff>